<commit_message>
Rebuild first-love exploration, answer feedback and romantic story scenes
</commit_message>
<xml_diff>
--- a/public/labs/first-love/first-love-template.xlsx
+++ b/public/labs/first-love/first-love-template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R3b6da01c96814bae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R616f4ea8f9524bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R8425917c8ed44a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R62c5fb9abb59421f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="Ree689debeb1242c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R7b4eeb2dbe124084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R152136fcc3ee4c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R525b8f1e07dc4678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="Rc98fee61450f4864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="Rd4562afd9c274a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R6957acac76fd4f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R9732286680f641fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -618,22 +618,22 @@
         <x:v>오늘은 미루지 않기로 했다</x:v>
       </x:c>
       <x:c r="E7" s="14" t="str">
-        <x:v>자료를 값이 작은 것부터 큰 순서로 놓으세요.</x:v>
+        <x:v>네 숫자를 작은 수부터 큰 수 순서로 놓으세요. 왼쪽이 가장 작은 수예요.</x:v>
       </x:c>
       <x:c r="F7" s="14" t="str">
-        <x:v>각자 한 장의 값을 알고 있습니다. 카드의 알파벳은 순서와 관계없습니다.</x:v>
+        <x:v>예: 3, −1, 2라면 −1 → 2 → 3 순서예요. 실제로 놓을 숫자는 아래 네 카드예요. A·B·C·D는 카드 이름이며 정답 순서가 아니에요.</x:v>
       </x:c>
       <x:c r="G7" s="14" t="str">
         <x:v>−7 &lt; −2 &lt; 0 &lt; 5이므로 C → A → D → B.</x:v>
       </x:c>
       <x:c r="H7" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>네 카드의 숫자를 서로 읽어 주세요. 알파벳은 이름일 뿐이에요.</x:v>
       </x:c>
       <x:c r="I7" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>음수 → 0 → 양수 순서예요. 음수끼리는 −9가 −1보다 작아요.</x:v>
       </x:c>
       <x:c r="J7" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>가장 작은 수의 카드를 누르고 1번째 칸을 누르세요. 같은 방법으로 네 칸을 채워요.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="104" customHeight="1">
@@ -650,7 +650,7 @@
         <x:v>같이 보던 책</x:v>
       </x:c>
       <x:c r="E8" s="14" t="str">
-        <x:v>책에 적힌 값을 계산해 알맞은 반납 칸과 연결하세요.</x:v>
+        <x:v>각 카드의 계산식을 풀고, 그 답이 적힌 칸에 놓으세요.</x:v>
       </x:c>
       <x:c r="F8" s="14" t="str">
         <x:v>네 칸에 책 한 권씩. 담당자는 책 안쪽 계산식을 읽어 주세요.</x:v>
@@ -659,13 +659,13 @@
         <x:v>A=5, B=−6, C=0, D=8.</x:v>
       </x:c>
       <x:c r="H8" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>담당 친구가 책에 적힌 계산식을 읽어 주세요.</x:v>
       </x:c>
       <x:c r="I8" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>먼저 식의 값을 구하고, 그 값이 적힌 반납 칸을 찾으세요.</x:v>
       </x:c>
       <x:c r="J8" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>카드를 누른 뒤 계산 결과가 적힌 칸을 누르세요. 네 칸에 한 장씩 놓아요.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="104" customHeight="1">
@@ -691,13 +691,13 @@
         <x:v>A·C·E·H는 짝수, B·D·F·G는 홀수.</x:v>
       </x:c>
       <x:c r="H9" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>각 친구가 두 숫자를 알려 주세요.</x:v>
       </x:c>
       <x:c r="I9" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>2로 나누어떨어지면 짝수예요. 음수도 분류할 수 있고 0도 짝수예요.</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>카드 → 짝수 또는 홀수 칸을 누르세요. 한 칸에 여러 장을 넣어도 돼요.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="104" customHeight="1">
@@ -714,22 +714,22 @@
         <x:v>수정본을 믿으면 안 되는 이유</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>옮겨 적은 각 항목을 유지하거나, 알맞은 설명 조각으로 수정하세요.</x:v>
+        <x:v>네 문장을 원본과 비교하세요. 같은 문장은 유지하고, 다른 문장은 원본대로 고치세요.</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
-        <x:v>원본은 자리별 기록에 있습니다. 수정할 항목에는 직접 올바른 설명을 골라 넣으세요.</x:v>
+        <x:v>왼쪽의 친구별 단서에 원본이 있어요. 문장 옆 선택 목록에서 “유지” 또는 올바른 수정 문장을 골라요.</x:v>
       </x:c>
       <x:c r="G10" s="14" t="str">
         <x:v>A·C는 유지. B는 F2, D는 F4로 수정.</x:v>
       </x:c>
       <x:c r="H10" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>왼쪽 단서에서 A·B·C·D의 원본을 각각 찾으세요.</x:v>
       </x:c>
       <x:c r="I10" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>지금 보이는 문장과 원본이 완전히 같으면 유지예요. 다른 문장만 고쳐요.</x:v>
       </x:c>
       <x:c r="J10" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>각 문장 옆 목록에서 유지를 고르거나 원본과 같은 수정 문장을 고르세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="104" customHeight="1">
@@ -737,7 +737,7 @@
         <x:v>P5</x:v>
       </x:c>
       <x:c r="B11" s="13" t="str">
-        <x:v>club</x:v>
+        <x:v>corridor</x:v>
       </x:c>
       <x:c r="C11" s="13" t="str">
         <x:v>route-match</x:v>
@@ -749,19 +749,19 @@
         <x:v>부호로 중간 지점을 정한 뒤, 절댓값 조건으로 도착함을 연결하세요.</x:v>
       </x:c>
       <x:c r="F11" s="14" t="str">
-        <x:v>1단계: 음수 → M1, 양수 → M2. 2단계: 각 지점의 안내에 따라 도착함을 정하세요. 두 단계를 모두 연결합니다.</x:v>
+        <x:v>① 부호로 음수 지점 / 양수 지점을 골라요. ② 각 친구가 가진 “절댓값 5 미만 / 5 이상” 안내로 도착함을 골라요. 카드마다 두 칸을 모두 채워요.</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
         <x:v>A: M1→T1, B: M2→T3, C: M1→T2, D: M2→T4.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>각 친구의 기록에는 자기 카드가 갈 두 번째 기준이 적혀 있어요.</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>음수는 음수 지점, 양수는 양수 지점으로 가요. 이어서 절댓값을 5와 비교해요.</x:v>
       </x:c>
       <x:c r="J11" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>카드마다 중간 지점과 도착함, 두 목록을 모두 골라 주세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="104" customHeight="1">
@@ -781,19 +781,19 @@
         <x:v>양수인 자료 네 장만 골라 작은 값부터 배열하세요.</x:v>
       </x:c>
       <x:c r="F12" s="14" t="str">
-        <x:v>각 자리에 두 장 중 한 장만 유효합니다. 확성기 같은 소품은 정답 기준이 아닙니다.</x:v>
+        <x:v>양수는 0보다 큰 수예요. 각 친구의 두 카드 중 하나씩 골라요. 음수 네 장은 위에 남겨 두세요.</x:v>
       </x:c>
       <x:c r="G12" s="14" t="str">
         <x:v>양수 C(2) → H(5) → B(7) → E(11).</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>각 친구가 두 장 중 양수 한 장을 골라 알려 주세요.</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>0보다 큰 네 값만 비교해요. 작은 수가 왼쪽이에요.</x:v>
       </x:c>
       <x:c r="J12" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>양수 네 장만 1~4번째 칸에 놓고, 음수 네 장은 위에 남겨 두세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="104" customHeight="1">
@@ -819,13 +819,13 @@
         <x:v>위쪽 B·C, 아래쪽 D·A.</x:v>
       </x:c>
       <x:c r="H13" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>한 카드에 대해 음수/양수와 홀수/짝수를 따로 판단하세요.</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>예를 들어 −10은 음수이면서 짝수예요. 두 기준에 모두 맞아야 해요.</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>카드 → 두 조건이 적힌 칸을 누르세요. 네 칸에 한 장씩 놓아요.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="104" customHeight="1">
@@ -833,7 +833,7 @@
         <x:v>P8</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
-        <x:v>club</x:v>
+        <x:v>corridor</x:v>
       </x:c>
       <x:c r="C14" s="13" t="str">
         <x:v>deduce</x:v>
@@ -845,19 +845,19 @@
         <x:v>네 조건을 모두 만족하는 후보 하나를 남기고, 나머지의 제외 근거를 표시하세요.</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>모든 후보를 가능 또는 제외로 옮깁니다. 제외할 때는 실제로 어긴 조건 번호 하나를 붙이세요.</x:v>
+        <x:v>후보마다 “가능” 또는 “제외”를 눌러요. 제외한 후보에는 어긴 조건 번호도 하나 골라요. 예: 양수라는 조건을 어긴 −2는 제외예요.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
         <x:v>네 조건을 모두 만족하는 수는 A의 6. B는 1, C는 2, D는 3, E는 4번 조건 때문에 제외한다. F·G·H도 조건 위반 근거를 하나씩 찾는다.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
-        <x:v>각자 받은 자료와 조건을 소리 내어 공유하세요.</x:v>
+        <x:v>친구 네 명의 조건을 차례로 읽어 주세요.</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>공통 기준을 자료 하나씩 적용하고 근거를 비교하세요.</x:v>
+        <x:v>조건 하나라도 어기면 제외예요. 예를 들어 −6은 양수 조건을 어겨요.</x:v>
       </x:c>
       <x:c r="J14" s="14" t="str">
-        <x:v>모든 자리를 채운 뒤 정답 확인을 누르세요. 움직이는 동안에는 오답이 늘지 않습니다.</x:v>
+        <x:v>여덟 후보 모두 가능/제외를 고르세요. 제외는 어긴 조건 하나도 선택하고, 가능은 하나만 남겨요.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -999,7 +999,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C7" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
         <x:v>−2</x:v>
@@ -1024,7 +1024,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>5</x:v>
@@ -1049,7 +1049,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
         <x:v>−7</x:v>
@@ -1074,7 +1074,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>0</x:v>
@@ -1099,7 +1099,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>−3 + 8</x:v>
@@ -1124,7 +1124,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>−4 − 2</x:v>
@@ -1149,7 +1149,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
         <x:v>7 − 7</x:v>
@@ -1174,7 +1174,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
         <x:v>2 × 4</x:v>
@@ -1199,7 +1199,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
         <x:v>−8</x:v>
@@ -1224,7 +1224,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
         <x:v>−3</x:v>
@@ -1249,7 +1249,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
         <x:v>0</x:v>
@@ -1274,7 +1274,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
         <x:v>5</x:v>
@@ -1299,7 +1299,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>자료 E</x:v>
+        <x:v>카드 E</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
         <x:v>12</x:v>
@@ -1324,7 +1324,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>자료 F</x:v>
+        <x:v>카드 F</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
         <x:v>−11</x:v>
@@ -1349,7 +1349,7 @@
         <x:v>G</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>자료 G</x:v>
+        <x:v>카드 G</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
         <x:v>7</x:v>
@@ -1374,7 +1374,7 @@
         <x:v>H</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>자료 H</x:v>
+        <x:v>카드 H</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
         <x:v>−2</x:v>
@@ -1399,7 +1399,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
         <x:v>절댓값은 0 이상이다.</x:v>
@@ -1426,7 +1426,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
         <x:v>−5는 −2보다 크다.</x:v>
@@ -1453,7 +1453,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
         <x:v>0은 양수도 음수도 아니다.</x:v>
@@ -1480,7 +1480,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
         <x:v>음수 두 개의 곱은 음수다.</x:v>
@@ -1507,7 +1507,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
         <x:v>−3</x:v>
@@ -1534,7 +1534,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
         <x:v>4</x:v>
@@ -1561,7 +1561,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
         <x:v>−6</x:v>
@@ -1588,7 +1588,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
         <x:v>5</x:v>
@@ -1615,7 +1615,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
         <x:v>−4</x:v>
@@ -1640,7 +1640,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
         <x:v>7</x:v>
@@ -1665,7 +1665,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
         <x:v>2</x:v>
@@ -1690,7 +1690,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
         <x:v>−9</x:v>
@@ -1715,7 +1715,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C35" s="9" t="str">
-        <x:v>자료 E</x:v>
+        <x:v>카드 E</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
         <x:v>11</x:v>
@@ -1740,7 +1740,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>자료 F</x:v>
+        <x:v>카드 F</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
         <x:v>−1</x:v>
@@ -1765,7 +1765,7 @@
         <x:v>G</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
-        <x:v>자료 G</x:v>
+        <x:v>카드 G</x:v>
       </x:c>
       <x:c r="D37" s="9" t="str">
         <x:v>−6</x:v>
@@ -1790,7 +1790,7 @@
         <x:v>H</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
-        <x:v>자료 H</x:v>
+        <x:v>카드 H</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
         <x:v>5</x:v>
@@ -1815,7 +1815,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C39" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D39" s="14" t="str">
         <x:v>6</x:v>
@@ -1840,7 +1840,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
         <x:v>−3</x:v>
@@ -1865,7 +1865,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C41" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D41" s="9" t="str">
         <x:v>−8</x:v>
@@ -1890,7 +1890,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
         <x:v>5</x:v>
@@ -1915,7 +1915,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C43" s="14" t="str">
-        <x:v>자료 A</x:v>
+        <x:v>카드 A</x:v>
       </x:c>
       <x:c r="D43" s="14" t="str">
         <x:v>6</x:v>
@@ -1942,7 +1942,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C44" s="9" t="str">
-        <x:v>자료 B</x:v>
+        <x:v>카드 B</x:v>
       </x:c>
       <x:c r="D44" s="9" t="str">
         <x:v>−6</x:v>
@@ -1969,7 +1969,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C45" s="9" t="str">
-        <x:v>자료 C</x:v>
+        <x:v>카드 C</x:v>
       </x:c>
       <x:c r="D45" s="9" t="str">
         <x:v>3</x:v>
@@ -1996,7 +1996,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C46" s="9" t="str">
-        <x:v>자료 D</x:v>
+        <x:v>카드 D</x:v>
       </x:c>
       <x:c r="D46" s="9" t="str">
         <x:v>12</x:v>
@@ -2023,7 +2023,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C47" s="9" t="str">
-        <x:v>자료 E</x:v>
+        <x:v>카드 E</x:v>
       </x:c>
       <x:c r="D47" s="9" t="str">
         <x:v>4</x:v>
@@ -2050,7 +2050,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C48" s="9" t="str">
-        <x:v>자료 F</x:v>
+        <x:v>카드 F</x:v>
       </x:c>
       <x:c r="D48" s="9" t="str">
         <x:v>−5</x:v>
@@ -2077,7 +2077,7 @@
         <x:v>G</x:v>
       </x:c>
       <x:c r="C49" s="9" t="str">
-        <x:v>자료 G</x:v>
+        <x:v>카드 G</x:v>
       </x:c>
       <x:c r="D49" s="9" t="str">
         <x:v>15</x:v>
@@ -2104,7 +2104,7 @@
         <x:v>H</x:v>
       </x:c>
       <x:c r="C50" s="9" t="str">
-        <x:v>자료 H</x:v>
+        <x:v>카드 H</x:v>
       </x:c>
       <x:c r="D50" s="9" t="str">
         <x:v>0</x:v>
@@ -2547,7 +2547,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D7" s="14" t="str">
         <x:v>내 기록은 −2. 음수는 0보다 작다.</x:v>
@@ -2561,7 +2561,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>내 기록은 5. 양수는 0보다 크다.</x:v>
@@ -2575,7 +2575,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
         <x:v>내 기록은 −7. 음수끼리는 절댓값이 클수록 작다.</x:v>
@@ -2589,7 +2589,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>내 기록은 0. 음수와 양수 사이에 놓는다.</x:v>
@@ -2603,7 +2603,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
         <x:v>A의 계산식은 −3 + 8이다.</x:v>
@@ -2617,7 +2617,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>B의 계산식은 −4 − 2이다.</x:v>
@@ -2631,7 +2631,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
         <x:v>C의 계산식은 7 − 7이다.</x:v>
@@ -2645,7 +2645,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
         <x:v>D의 계산식은 2 × 4이다.</x:v>
@@ -2659,7 +2659,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
         <x:v>A=−8, B=−3. 나머지가 0이면 짝수다.</x:v>
@@ -2673,7 +2673,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
         <x:v>C=0, D=5. 0도 짝수다.</x:v>
@@ -2687,7 +2687,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
         <x:v>E=12, F=−11. 부호와 홀짝은 별개다.</x:v>
@@ -2701,7 +2701,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
         <x:v>G=7, H=−2. 음수도 2로 나눌 수 있다.</x:v>
@@ -2715,7 +2715,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C19" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D19" s="14" t="str">
         <x:v>A 원본: 절댓값은 0 이상이다.</x:v>
@@ -2729,7 +2729,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
         <x:v>B 원본: −5는 −2보다 작다.</x:v>
@@ -2743,7 +2743,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
         <x:v>C 원본: 0은 양수도 음수도 아니다.</x:v>
@@ -2757,7 +2757,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
         <x:v>D 원본: 음수 두 개의 곱은 양수다.</x:v>
@@ -2771,7 +2771,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C23" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D23" s="14" t="str">
         <x:v>A=−3. M1에서 절댓값 5 미만 → 봉투함.</x:v>
@@ -2785,7 +2785,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
         <x:v>B=4. M2에서 절댓값 5 미만 → 반납함.</x:v>
@@ -2799,7 +2799,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
         <x:v>C=−6. M1에서 절댓값 5 이상 → 기록함.</x:v>
@@ -2813,7 +2813,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
         <x:v>D=5. M2에서 절댓값 5 이상 → 자료함.</x:v>
@@ -2827,7 +2827,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C27" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D27" s="14" t="str">
         <x:v>A=−4, B=7. 양수인 한 장만 남긴다.</x:v>
@@ -2841,7 +2841,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
         <x:v>C=2, D=−9. 0보다 큰 값을 고른다.</x:v>
@@ -2855,7 +2855,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
         <x:v>E=11, F=−1. 내 유효한 값은 다른 자리와 비교한다.</x:v>
@@ -2869,7 +2869,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
         <x:v>G=−6, H=5. 선택한 네 값은 오름차순으로 놓는다.</x:v>
@@ -2883,7 +2883,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C31" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D31" s="14" t="str">
         <x:v>A=6. 부호와 홀짝을 각각 확인한다.</x:v>
@@ -2897,7 +2897,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
         <x:v>B=−3. 음수 중에서도 홀수와 짝수가 나뉜다.</x:v>
@@ -2911,7 +2911,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
         <x:v>C=−8. 음수의 짝수는 오른쪽 위다.</x:v>
@@ -2925,7 +2925,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
         <x:v>D=5. 양수의 홀수는 왼쪽 아래다.</x:v>
@@ -2939,7 +2939,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C35" s="14" t="str">
-        <x:v>1번의 기록</x:v>
+        <x:v>1번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D35" s="14" t="str">
         <x:v>조건 1: 값은 0보다 큰 양수다.</x:v>
@@ -2953,7 +2953,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>2번의 기록</x:v>
+        <x:v>2번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
         <x:v>조건 2: 값은 짝수다.</x:v>
@@ -2967,7 +2967,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
-        <x:v>3번의 기록</x:v>
+        <x:v>3번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D37" s="9" t="str">
         <x:v>조건 3: 절댓값은 10보다 작다.</x:v>
@@ -2981,7 +2981,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
-        <x:v>4번의 기록</x:v>
+        <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
         <x:v>조건 4: 값은 3의 배수다.</x:v>

</xml_diff>

<commit_message>
Add scene expressions, event accident story and multiple valid P8 reasons
</commit_message>
<xml_diff>
--- a/public/labs/first-love/first-love-template.xlsx
+++ b/public/labs/first-love/first-love-template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R152136fcc3ee4c18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R525b8f1e07dc4678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="Rc98fee61450f4864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="Rd4562afd9c274a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R6957acac76fd4f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R9732286680f641fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="Rc8818b1db0564e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="Rc9d803832d684997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="Rb5f38c3cfcec4807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R21736e69a3074db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="Rfc447fb98a4c4048"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R3c0357185efe48ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -828,7 +828,7 @@
         <x:v>카드 → 두 조건이 적힌 칸을 누르세요. 네 칸에 한 장씩 놓아요.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="104" customHeight="1">
+    <x:row r="14" ht="165" customHeight="1">
       <x:c r="A14" s="13" t="str">
         <x:v>P8</x:v>
       </x:c>
@@ -845,10 +845,10 @@
         <x:v>네 조건을 모두 만족하는 후보 하나를 남기고, 나머지의 제외 근거를 표시하세요.</x:v>
       </x:c>
       <x:c r="F14" s="14" t="str">
-        <x:v>후보마다 “가능” 또는 “제외”를 눌러요. 제외한 후보에는 어긴 조건 번호도 하나 골라요. 예: 양수라는 조건을 어긴 −2는 제외예요.</x:v>
+        <x:v>후보마다 “가능” 또는 “제외”를 눌러요. 제외한 후보에는 어긴 조건 번호를 하나 이상 골라요. 여러 번호를 고르면 모두 맞는 근거여야 해요. 예: 양수라는 조건을 어긴 −2는 제외예요.</x:v>
       </x:c>
       <x:c r="G14" s="14" t="str">
-        <x:v>네 조건을 모두 만족하는 수는 A의 6. B는 1, C는 2, D는 3, E는 4번 조건 때문에 제외한다. F·G·H도 조건 위반 근거를 하나씩 찾는다.</x:v>
+        <x:v>네 조건을 모두 만족하는 수는 A의 6. B는 1, C는 2, D는 3, E는 4번 조건 때문에 제외한다. F는 1·2·4번, G는 2·3번, H(0)는 1·4번을 어긴다. 이 중 하나 또는 여러 개를 골라도 인정한다. 0은 짝수이며 절댓값이 10보다 작다. 조건 4에서는 0을 명시적으로 제외했다.</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
         <x:v>친구 네 명의 조건을 차례로 읽어 주세요.</x:v>
@@ -2118,7 +2118,7 @@
       <x:c r="G50" s="10" t="str"/>
       <x:c r="H50" s="10" t="str"/>
       <x:c r="I50" s="9" t="str">
-        <x:v>2|3|4</x:v>
+        <x:v>2|3</x:v>
       </x:c>
       <x:c r="J50" s="9" t="str"/>
       <x:c r="K50" s="9" t="str"/>
@@ -2973,7 +2973,7 @@
         <x:v>조건 3: 절댓값은 10보다 작다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="52" customHeight="1">
+    <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="10" t="str">
         <x:v>P8</x:v>
       </x:c>
@@ -2984,7 +2984,7 @@
         <x:v>4번 친구가 읽어 줄 내용</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
-        <x:v>조건 4: 값은 3의 배수다.</x:v>
+        <x:v>조건 4: 값은 0이 아닌 3의 배수다. (예: −6, −3, 3, 6)</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Halve first-love ending wrong-answer thresholds
Use smile through 5 wrong answers, surprise from 6 through 14 (including 10), and disgust from 15. Update teacher defaults, workbook, authoring prompt, guide, and browser module versions together. Existing class snapshots and saved endings remain unchanged.

Validation: 17 first-love tests passed, including ending boundaries, frozen endings, and six-sheet XLSX round trip. Workbook cell changes are limited to settings B12 and B13.
</commit_message>
<xml_diff>
--- a/public/labs/first-love/first-love-template.xlsx
+++ b/public/labs/first-love/first-love-template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="Rc8818b1db0564e7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="Rc9d803832d684997"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="Rb5f38c3cfcec4807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R21736e69a3074db6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="Rfc447fb98a4c4048"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R3c0357185efe48ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="Rf9ee8d6d3dd24e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R2aca30f6883e4664"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="Red436e0bfa524f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R888de6abb62b495a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R3b0edd29fea945ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="Rfac62aec5d714910"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -465,7 +465,7 @@
         <x:v>미소_최대오답</x:v>
       </x:c>
       <x:c r="B12" s="15" t="n">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C12" s="13" t="str">
         <x:v>시작한 수업에는 고정</x:v>
@@ -476,7 +476,7 @@
         <x:v>당황_최대오답</x:v>
       </x:c>
       <x:c r="B13" s="15" t="n">
-        <x:v>29</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C13" s="13" t="str">
         <x:v>그보다 많으면 부정 표정</x:v>

</xml_diff>